<commit_message>
region grid: San Antonio
</commit_message>
<xml_diff>
--- a/region/San-Antonio-overview-grid.xlsx
+++ b/region/San-Antonio-overview-grid.xlsx
@@ -112,7 +112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD61"/>
+  <dimension ref="A1:AD62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -150,7 +150,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">H-E-B  |  Region Overview information — San Antonio — generated 8/17/2026</t>
+          <t xml:space="preserve">H-E-B  |  Region Overview information — San Antonio — generated 8/28/2026</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       <c r="N33" s="5"/>
       <c r="O33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">12’3' x 24’6'</t>
+          <t xml:space="preserve">12'3" x 24'6"</t>
         </is>
       </c>
       <c r="P33" s="5"/>
@@ -5738,7 +5738,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">TX46B</t>
+          <t xml:space="preserve">TX39A</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
@@ -5746,16 +5746,8 @@
           <t xml:space="preserve">MH Outdoor Media</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Brandon Wilburn</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bwilburn@machaik.com</t>
-        </is>
-      </c>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
       <c r="E57" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">San Antonio</t>
@@ -5763,44 +5755,44 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Static Bulletin</t>
+          <t xml:space="preserve">Bulletin</t>
         </is>
       </c>
       <c r="G57" s="5"/>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/S of Hwy 90 Bus., 600 feet E/o FM 725.    Seguin, Texas N/S, W/F</t>
+          <t xml:space="preserve">N/S of IH-10 East, .7 Miles E/o Loop 1604.     Exit 587, E/F</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seguin</t>
+          <t xml:space="preserve">San Antonio</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">78155</t>
+          <t xml:space="preserve">78230</t>
         </is>
       </c>
       <c r="K57" s="11">
-        <v>29.555712</v>
+        <v>29.469312</v>
       </c>
       <c r="L57" s="11">
-        <v>-98.027557</v>
+        <v>-98.281866</v>
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">West</t>
+          <t xml:space="preserve">E/F</t>
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Left</t>
+          <t xml:space="preserve">Right</t>
         </is>
       </c>
       <c r="O57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">10' x 30'</t>
+          <t xml:space="preserve">14'0x48'0</t>
         </is>
       </c>
       <c r="P57" s="5" t="inlineStr">
@@ -5810,32 +5802,28 @@
       </c>
       <c r="Q57" s="5"/>
       <c r="R57" s="7">
-        <v>46258</v>
+        <v>46398</v>
       </c>
       <c r="S57" s="7">
-        <v>46299</v>
+        <v>46761</v>
       </c>
       <c r="T57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">MH Outdoor 15551-1 TX46B Seguin HEB-SIGNED 8-12-26 (awaiting MH signature).pdf</t>
+          <t xml:space="preserve">MH Outdoor 15491-4 TX39A HEB-SIGNED 8-26-26 (awaiting MH signature).pdf</t>
         </is>
       </c>
       <c r="U57" s="5">
-        <v>166460</v>
+        <v>1536325</v>
       </c>
       <c r="V57" s="9">
-        <v>550</v>
+        <v>1200</v>
       </c>
       <c r="W57" s="9"/>
       <c r="X57" s="5"/>
       <c r="Y57" s="5">
-        <v>5</v>
-      </c>
-      <c r="Z57" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">📐 Spec Sheet</t>
-        </is>
-      </c>
+        <v>4.7</v>
+      </c>
+      <c r="Z57" s="5"/>
       <c r="AA57" s="5"/>
       <c r="AB57" s="5"/>
       <c r="AC57" s="7"/>
@@ -5844,22 +5832,22 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NT #1302</t>
+          <t xml:space="preserve">TX46B</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">New Tradition</t>
+          <t xml:space="preserve">MH Outdoor Media</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jill Maugle</t>
+          <t xml:space="preserve">Brandon Wilburn</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">jill@newtradition.com</t>
+          <t xml:space="preserve">bwilburn@machaik.com</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -5869,61 +5857,73 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Place-Based - Banners ✨</t>
+          <t xml:space="preserve">Static Bulletin</t>
         </is>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Riverwalk – Rivercenter: Banners</t>
+          <t xml:space="preserve">N/S of Hwy 90 Bus., 600 feet E/o FM 725.    Seguin, Texas N/S, W/F</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">San Antonio</t>
-        </is>
-      </c>
-      <c r="J58" s="4"/>
+          <t xml:space="preserve">Seguin</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78155</t>
+        </is>
+      </c>
       <c r="K58" s="10">
-        <v>29.423867</v>
+        <v>29.555712</v>
       </c>
       <c r="L58" s="10">
-        <v>-98.485107</v>
-      </c>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
+        <v>-98.027557</v>
+      </c>
+      <c r="M58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">West</t>
+        </is>
+      </c>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Left</t>
+        </is>
+      </c>
       <c r="O58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">25' H x 10' W Sky Murals (2) ~ 12' H x 2' 6" W Trumpet Banners (10)</t>
-        </is>
-      </c>
-      <c r="P58" s="4"/>
-      <c r="Q58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New Tradition — Media #1302 Riverwalk/Rivercenter banners (12 units), San Antonio, 8/24–11/1/26, $94,172 — HEB-SIGNED 8/12/26, awaiting NT Credit Dept</t>
-        </is>
-      </c>
+          <t xml:space="preserve">10' x 30'</t>
+        </is>
+      </c>
+      <c r="P58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="Q58" s="4"/>
       <c r="R58" s="6">
         <v>46258</v>
       </c>
       <c r="S58" s="6">
-        <v>46327</v>
+        <v>46299</v>
       </c>
       <c r="T58" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">New Tradition 1302 San Antonio HEB-SIGNED 8-12-26 (awaiting NT Credit Dept).pdf</t>
+          <t xml:space="preserve">MH Outdoor 15551-1 TX46B Seguin HEB-SIGNED 8-12-26 (awaiting MH signature).pdf</t>
         </is>
       </c>
       <c r="U58" s="4">
-        <v>2448716</v>
+        <v>166460</v>
       </c>
       <c r="V58" s="8">
-        <v>31186</v>
+        <v>550</v>
       </c>
       <c r="W58" s="8"/>
       <c r="X58" s="4"/>
       <c r="Y58" s="4">
-        <v>0.7</v>
+        <v>5</v>
       </c>
       <c r="Z58" s="12" t="inlineStr">
         <is>
@@ -5938,22 +5938,22 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">02_6069O</t>
+          <t xml:space="preserve">NT #1302</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outfront Media</t>
+          <t xml:space="preserve">New Tradition</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sammy Tamporello</t>
+          <t xml:space="preserve">Jill Maugle</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">sammy.tamporello@outfront.com</t>
+          <t xml:space="preserve">jill@newtradition.com</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -5963,88 +5963,76 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bulletin</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">535952</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Place-Based - Banners ✨</t>
+        </is>
+      </c>
+      <c r="G59" s="5"/>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">US 281 N .5M S/O Airport Blvd/Loop 410 ES F/N F/N</t>
-        </is>
-      </c>
-      <c r="I59" s="5"/>
+          <t xml:space="preserve">Riverwalk – Rivercenter: Banners</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">San Antonio</t>
+        </is>
+      </c>
       <c r="J59" s="5"/>
       <c r="K59" s="11">
-        <v>29.51194</v>
+        <v>29.423867</v>
       </c>
       <c r="L59" s="11">
-        <v>-98.47541</v>
-      </c>
-      <c r="M59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">North</t>
-        </is>
-      </c>
+        <v>-98.485107</v>
+      </c>
+      <c r="M59" s="5"/>
       <c r="N59" s="5"/>
       <c r="O59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">14' x 48'</t>
+          <t xml:space="preserve">25' H x 10' W Sky Murals (2) ~ 12' H x 2' 6" W Trumpet Banners (10)</t>
         </is>
       </c>
       <c r="P59" s="5"/>
       <c r="Q59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">281 HV</t>
+          <t xml:space="preserve">New Tradition — Media #1302 Riverwalk/Rivercenter banners (12 units), San Antonio, 8/24–11/1/26, $94,172 — HEB-SIGNED 8/12/26, awaiting NT Credit Dept</t>
         </is>
       </c>
       <c r="R59" s="7">
-        <v>46209</v>
+        <v>46258</v>
       </c>
       <c r="S59" s="7">
-        <v>46439</v>
+        <v>46327</v>
       </c>
       <c r="T59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charli Sowrey_encrypted_.pdf</t>
+          <t xml:space="preserve">New Tradition 1302 San Antonio HEB-SIGNED 8-12-26 (awaiting NT Credit Dept).pdf</t>
         </is>
       </c>
       <c r="U59" s="5">
-        <v>432834</v>
+        <v>2448716</v>
       </c>
       <c r="V59" s="9">
-        <v>7137</v>
+        <v>31186</v>
       </c>
       <c r="W59" s="9"/>
       <c r="X59" s="5"/>
       <c r="Y59" s="5">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="Z59" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">📐 Spec Sheet</t>
         </is>
       </c>
-      <c r="AA59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">More Dinner. Less Dinero.</t>
-        </is>
-      </c>
+      <c r="AA59" s="5"/>
       <c r="AB59" s="5"/>
       <c r="AC59" s="7"/>
-      <c r="AD59" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cowboys: Dak</t>
-        </is>
-      </c>
+      <c r="AD59" s="5"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2_1963F</t>
+          <t xml:space="preserve">02_6069O</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -6069,30 +6057,26 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Digital Bulletin</t>
+          <t xml:space="preserve">Bulletin</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">50769131</t>
+          <t xml:space="preserve">535952</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NW Loop 410 W/O Bandera Rd. F/N F/N</t>
+          <t xml:space="preserve">US 281 N .5M S/O Airport Blvd/Loop 410 ES F/N F/N</t>
         </is>
       </c>
       <c r="I60" s="4"/>
-      <c r="J60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">78238</t>
-        </is>
-      </c>
+      <c r="J60" s="4"/>
       <c r="K60" s="10">
-        <v>29.48264</v>
+        <v>29.51194</v>
       </c>
       <c r="L60" s="10">
-        <v>-98.602335</v>
+        <v>-98.47541</v>
       </c>
       <c r="M60" s="4" t="inlineStr">
         <is>
@@ -6102,56 +6086,76 @@
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">14'x48'</t>
+          <t xml:space="preserve">14' x 48'</t>
         </is>
       </c>
       <c r="P60" s="4"/>
-      <c r="Q60" s="4"/>
+      <c r="Q60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">281 HV</t>
+        </is>
+      </c>
       <c r="R60" s="6">
-        <v>46258</v>
+        <v>46209</v>
       </c>
       <c r="S60" s="6">
-        <v>46327</v>
+        <v>46439</v>
       </c>
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outfront 4491743 2_1963 SA Digital Bulletin HEB-SIGNED 8-13-26 (awaiting Outfront GM).pdf</t>
+          <t xml:space="preserve">Charli Sowrey_encrypted_.pdf</t>
         </is>
       </c>
       <c r="U60" s="4">
-        <v>1522800</v>
+        <v>432834</v>
       </c>
       <c r="V60" s="8">
-        <v>3500</v>
+        <v>7137</v>
       </c>
       <c r="W60" s="8"/>
       <c r="X60" s="4"/>
       <c r="Y60" s="4">
-        <v>0.5</v>
+        <v>1.1</v>
       </c>
       <c r="Z60" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">📐 Spec Sheet</t>
         </is>
       </c>
-      <c r="AA60" s="4"/>
+      <c r="AA60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">More Dinner. Less Dinero.</t>
+        </is>
+      </c>
       <c r="AB60" s="4"/>
       <c r="AC60" s="6"/>
-      <c r="AD60" s="4"/>
+      <c r="AD60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cowboys: Dak</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">54560.2</t>
+          <t xml:space="preserve">2_1963F</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">SignAd</t>
-        </is>
-      </c>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
+          <t xml:space="preserve">Outfront Media</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sammy Tamporello</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sammy.tamporello@outfront.com</t>
+        </is>
+      </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">San Antonio</t>
@@ -6162,48 +6166,40 @@
           <t xml:space="preserve">Digital Bulletin</t>
         </is>
       </c>
-      <c r="G61" s="5"/>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50769131</t>
+        </is>
+      </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">FM 78/OLD SEGUIN RD/.7 MI E/O WALZEM RD/CONVERSE-LED-LH/WB</t>
-        </is>
-      </c>
-      <c r="I61" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONVERSE</t>
-        </is>
-      </c>
+          <t xml:space="preserve">NW Loop 410 W/O Bandera Rd. F/N F/N</t>
+        </is>
+      </c>
+      <c r="I61" s="5"/>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">78109</t>
+          <t xml:space="preserve">78238</t>
         </is>
       </c>
       <c r="K61" s="11">
-        <v>29.4964</v>
+        <v>29.48264</v>
       </c>
       <c r="L61" s="11">
-        <v>-98.3239</v>
+        <v>-98.602335</v>
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">East</t>
-        </is>
-      </c>
-      <c r="N61" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Left</t>
-        </is>
-      </c>
+          <t xml:space="preserve">North</t>
+        </is>
+      </c>
+      <c r="N61" s="5"/>
       <c r="O61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">10 ft x 36 ft</t>
-        </is>
-      </c>
-      <c r="P61" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Y</t>
-        </is>
-      </c>
+          <t xml:space="preserve">14'x48'</t>
+        </is>
+      </c>
+      <c r="P61" s="5"/>
       <c r="Q61" s="5"/>
       <c r="R61" s="7">
         <v>46258</v>
@@ -6213,19 +6209,19 @@
       </c>
       <c r="T61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">SignAd 052630 54560.2 Converse LED HEB-SIGNED 8-12-26 (awaiting SignAd officer).pdf</t>
+          <t xml:space="preserve">Outfront 4491743 2_1963 SA Digital Bulletin HEB-SIGNED 8-13-26 (awaiting Outfront GM).pdf</t>
         </is>
       </c>
       <c r="U61" s="5">
-        <v>24119</v>
+        <v>1522800</v>
       </c>
       <c r="V61" s="9">
-        <v>1000</v>
+        <v>3500</v>
       </c>
       <c r="W61" s="9"/>
       <c r="X61" s="5"/>
       <c r="Y61" s="5">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="Z61" s="13" t="inlineStr">
         <is>
@@ -6236,6 +6232,104 @@
       <c r="AB61" s="5"/>
       <c r="AC61" s="7"/>
       <c r="AD61" s="5"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">54560.2</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SignAd</t>
+        </is>
+      </c>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">San Antonio</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Digital Bulletin</t>
+        </is>
+      </c>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FM 78/OLD SEGUIN RD/.7 MI E/O WALZEM RD/CONVERSE-LED-LH/WB</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONVERSE</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78109</t>
+        </is>
+      </c>
+      <c r="K62" s="10">
+        <v>29.4964</v>
+      </c>
+      <c r="L62" s="10">
+        <v>-98.3239</v>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">East</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Left</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 ft x 36 ft</t>
+        </is>
+      </c>
+      <c r="P62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="Q62" s="4"/>
+      <c r="R62" s="6">
+        <v>46258</v>
+      </c>
+      <c r="S62" s="6">
+        <v>46327</v>
+      </c>
+      <c r="T62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SignAd 052630 54560.2 Converse LED HEB-SIGNED 8-12-26 (awaiting SignAd officer).pdf</t>
+        </is>
+      </c>
+      <c r="U62" s="4">
+        <v>24119</v>
+      </c>
+      <c r="V62" s="8">
+        <v>1000</v>
+      </c>
+      <c r="W62" s="8"/>
+      <c r="X62" s="4"/>
+      <c r="Y62" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="Z62" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">📐 Spec Sheet</t>
+        </is>
+      </c>
+      <c r="AA62" s="4"/>
+      <c r="AB62" s="4"/>
+      <c r="AC62" s="6"/>
+      <c r="AD62" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:AD3"/>
@@ -6288,11 +6382,11 @@
     <hyperlink ref="Z52" r:id="rIdH42"/>
     <hyperlink ref="Z55" r:id="rIdH43"/>
     <hyperlink ref="Z56" r:id="rIdH44"/>
-    <hyperlink ref="Z57" r:id="rIdH45"/>
-    <hyperlink ref="Z58" r:id="rIdH46"/>
-    <hyperlink ref="Z59" r:id="rIdH47"/>
-    <hyperlink ref="Z60" r:id="rIdH48"/>
-    <hyperlink ref="Z61" r:id="rIdH49"/>
+    <hyperlink ref="Z58" r:id="rIdH45"/>
+    <hyperlink ref="Z59" r:id="rIdH46"/>
+    <hyperlink ref="Z60" r:id="rIdH47"/>
+    <hyperlink ref="Z61" r:id="rIdH48"/>
+    <hyperlink ref="Z62" r:id="rIdH49"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>